<commit_message>
Export SAM segmented cutouts
</commit_message>
<xml_diff>
--- a/report/sam_results/sam_instance_stats.xlsx
+++ b/report/sam_results/sam_instance_stats.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J20"/>
+  <dimension ref="A1:J18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -648,7 +648,7 @@
         <v>0.804</v>
       </c>
       <c r="C7" t="n">
-        <v>14879</v>
+        <v>16611</v>
       </c>
       <c r="D7" t="n">
         <v>744</v>
@@ -657,434 +657,370 @@
         <v>688</v>
       </c>
       <c r="F7" t="n">
-        <v>124</v>
+        <v>131</v>
       </c>
       <c r="G7" t="n">
-        <v>186</v>
+        <v>201</v>
       </c>
       <c r="H7" t="n">
-        <v>209.2</v>
+        <v>206.1</v>
       </c>
       <c r="I7" t="n">
-        <v>156.4</v>
+        <v>152</v>
       </c>
       <c r="J7" t="n">
-        <v>59.8</v>
+        <v>55.4</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B8" t="n">
-        <v>0.8053</v>
+        <v>0.8574000000000001</v>
       </c>
       <c r="C8" t="n">
-        <v>17471</v>
+        <v>17089</v>
       </c>
       <c r="D8" t="n">
-        <v>168</v>
+        <v>336</v>
       </c>
       <c r="E8" t="n">
         <v>800</v>
       </c>
       <c r="F8" t="n">
-        <v>169</v>
+        <v>145</v>
       </c>
       <c r="G8" t="n">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="H8" t="n">
-        <v>169.6</v>
+        <v>179.5</v>
       </c>
       <c r="I8" t="n">
-        <v>119.2</v>
+        <v>128.2</v>
       </c>
       <c r="J8" t="n">
-        <v>29</v>
+        <v>30.3</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B9" t="n">
-        <v>0.8375</v>
+        <v>0.8538</v>
       </c>
       <c r="C9" t="n">
-        <v>17088</v>
+        <v>14872</v>
       </c>
       <c r="D9" t="n">
-        <v>336</v>
+        <v>521</v>
       </c>
       <c r="E9" t="n">
-        <v>800</v>
+        <v>824</v>
       </c>
       <c r="F9" t="n">
-        <v>145</v>
+        <v>140</v>
       </c>
       <c r="G9" t="n">
-        <v>157</v>
+        <v>129</v>
       </c>
       <c r="H9" t="n">
-        <v>170.8</v>
+        <v>169.2</v>
       </c>
       <c r="I9" t="n">
-        <v>122.5</v>
+        <v>123</v>
       </c>
       <c r="J9" t="n">
-        <v>29.6</v>
+        <v>30</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B10" t="n">
-        <v>0.7765</v>
+        <v>0.8391</v>
       </c>
       <c r="C10" t="n">
-        <v>3053</v>
+        <v>12561</v>
       </c>
       <c r="D10" t="n">
-        <v>525</v>
+        <v>651</v>
       </c>
       <c r="E10" t="n">
-        <v>910</v>
+        <v>801</v>
       </c>
       <c r="F10" t="n">
-        <v>126</v>
+        <v>130</v>
       </c>
       <c r="G10" t="n">
-        <v>45</v>
+        <v>132</v>
       </c>
       <c r="H10" t="n">
-        <v>55.2</v>
+        <v>192.6</v>
       </c>
       <c r="I10" t="n">
-        <v>42.1</v>
+        <v>137</v>
       </c>
       <c r="J10" t="n">
-        <v>21.4</v>
+        <v>29.2</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B11" t="n">
-        <v>0.8257</v>
+        <v>0.8088</v>
       </c>
       <c r="C11" t="n">
-        <v>17955</v>
+        <v>2105</v>
       </c>
       <c r="D11" t="n">
-        <v>636</v>
+        <v>847</v>
       </c>
       <c r="E11" t="n">
-        <v>800</v>
+        <v>811</v>
       </c>
       <c r="F11" t="n">
-        <v>145</v>
+        <v>46</v>
       </c>
       <c r="G11" t="n">
-        <v>153</v>
+        <v>64</v>
       </c>
       <c r="H11" t="n">
-        <v>164.6</v>
+        <v>210.5</v>
       </c>
       <c r="I11" t="n">
-        <v>117.4</v>
+        <v>149.2</v>
       </c>
       <c r="J11" t="n">
-        <v>26.2</v>
+        <v>52.4</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B12" t="n">
-        <v>0.8132</v>
+        <v>0.8333</v>
       </c>
       <c r="C12" t="n">
-        <v>13017</v>
+        <v>4979</v>
       </c>
       <c r="D12" t="n">
-        <v>775</v>
+        <v>904</v>
       </c>
       <c r="E12" t="n">
-        <v>817</v>
+        <v>809</v>
       </c>
       <c r="F12" t="n">
-        <v>138</v>
+        <v>116</v>
       </c>
       <c r="G12" t="n">
-        <v>138</v>
+        <v>72</v>
       </c>
       <c r="H12" t="n">
-        <v>150.5</v>
+        <v>187.4</v>
       </c>
       <c r="I12" t="n">
-        <v>104.4</v>
+        <v>139.9</v>
       </c>
       <c r="J12" t="n">
-        <v>22.2</v>
+        <v>77</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="B13" t="n">
-        <v>0.8199</v>
+        <v>0.9306</v>
       </c>
       <c r="C13" t="n">
-        <v>11009</v>
+        <v>12674</v>
       </c>
       <c r="D13" t="n">
-        <v>900</v>
+        <v>48</v>
       </c>
       <c r="E13" t="n">
-        <v>809</v>
+        <v>1036</v>
       </c>
       <c r="F13" t="n">
-        <v>145</v>
+        <v>134</v>
       </c>
       <c r="G13" t="n">
-        <v>144</v>
+        <v>126</v>
       </c>
       <c r="H13" t="n">
-        <v>135.9</v>
+        <v>191.4</v>
       </c>
       <c r="I13" t="n">
-        <v>98.8</v>
+        <v>99.7</v>
       </c>
       <c r="J13" t="n">
-        <v>36.8</v>
+        <v>28.4</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="B14" t="n">
-        <v>0.8609</v>
+        <v>0.9549</v>
       </c>
       <c r="C14" t="n">
-        <v>10157</v>
+        <v>17842</v>
       </c>
       <c r="D14" t="n">
-        <v>1044</v>
+        <v>240</v>
       </c>
       <c r="E14" t="n">
-        <v>864</v>
+        <v>1024</v>
       </c>
       <c r="F14" t="n">
-        <v>145</v>
+        <v>159</v>
       </c>
       <c r="G14" t="n">
-        <v>86</v>
+        <v>135</v>
       </c>
       <c r="H14" t="n">
-        <v>126.2</v>
+        <v>209.2</v>
       </c>
       <c r="I14" t="n">
-        <v>86.40000000000001</v>
+        <v>125.3</v>
       </c>
       <c r="J14" t="n">
-        <v>18.3</v>
+        <v>42</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="B15" t="n">
-        <v>0.9306</v>
+        <v>0.9175</v>
       </c>
       <c r="C15" t="n">
-        <v>12674</v>
+        <v>18686</v>
       </c>
       <c r="D15" t="n">
-        <v>48</v>
+        <v>432</v>
       </c>
       <c r="E15" t="n">
-        <v>1036</v>
+        <v>1024</v>
       </c>
       <c r="F15" t="n">
-        <v>134</v>
+        <v>147</v>
       </c>
       <c r="G15" t="n">
-        <v>126</v>
+        <v>157</v>
       </c>
       <c r="H15" t="n">
-        <v>191.4</v>
+        <v>203.2</v>
       </c>
       <c r="I15" t="n">
-        <v>99.7</v>
+        <v>124.9</v>
       </c>
       <c r="J15" t="n">
-        <v>28.4</v>
+        <v>37.5</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="B16" t="n">
-        <v>0.9549</v>
+        <v>0.929</v>
       </c>
       <c r="C16" t="n">
-        <v>17842</v>
+        <v>14225</v>
       </c>
       <c r="D16" t="n">
-        <v>240</v>
+        <v>612</v>
       </c>
       <c r="E16" t="n">
         <v>1024</v>
       </c>
       <c r="F16" t="n">
-        <v>159</v>
+        <v>164</v>
       </c>
       <c r="G16" t="n">
-        <v>135</v>
+        <v>119</v>
       </c>
       <c r="H16" t="n">
         <v>209.2</v>
       </c>
       <c r="I16" t="n">
-        <v>125.3</v>
+        <v>129.3</v>
       </c>
       <c r="J16" t="n">
-        <v>42</v>
+        <v>41.6</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="B17" t="n">
-        <v>0.9175</v>
+        <v>0.907</v>
       </c>
       <c r="C17" t="n">
-        <v>18686</v>
+        <v>14336</v>
       </c>
       <c r="D17" t="n">
-        <v>432</v>
+        <v>792</v>
       </c>
       <c r="E17" t="n">
         <v>1024</v>
       </c>
       <c r="F17" t="n">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="G17" t="n">
-        <v>157</v>
+        <v>126</v>
       </c>
       <c r="H17" t="n">
-        <v>203.2</v>
+        <v>206.7</v>
       </c>
       <c r="I17" t="n">
-        <v>124.9</v>
+        <v>129.6</v>
       </c>
       <c r="J17" t="n">
-        <v>37.5</v>
+        <v>44.3</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="B18" t="n">
-        <v>0.929</v>
+        <v>0.7989000000000001</v>
       </c>
       <c r="C18" t="n">
-        <v>14225</v>
+        <v>12104</v>
       </c>
       <c r="D18" t="n">
-        <v>612</v>
+        <v>983</v>
       </c>
       <c r="E18" t="n">
         <v>1024</v>
       </c>
       <c r="F18" t="n">
-        <v>164</v>
+        <v>112</v>
       </c>
       <c r="G18" t="n">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="H18" t="n">
-        <v>209.2</v>
+        <v>204.4</v>
       </c>
       <c r="I18" t="n">
-        <v>129.3</v>
+        <v>125.2</v>
       </c>
       <c r="J18" t="n">
-        <v>41.6</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="n">
-        <v>19</v>
-      </c>
-      <c r="B19" t="n">
-        <v>0.907</v>
-      </c>
-      <c r="C19" t="n">
-        <v>14336</v>
-      </c>
-      <c r="D19" t="n">
-        <v>792</v>
-      </c>
-      <c r="E19" t="n">
-        <v>1024</v>
-      </c>
-      <c r="F19" t="n">
-        <v>145</v>
-      </c>
-      <c r="G19" t="n">
-        <v>126</v>
-      </c>
-      <c r="H19" t="n">
-        <v>206.7</v>
-      </c>
-      <c r="I19" t="n">
-        <v>129.6</v>
-      </c>
-      <c r="J19" t="n">
-        <v>44.3</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="n">
-        <v>20</v>
-      </c>
-      <c r="B20" t="n">
-        <v>0.7989000000000001</v>
-      </c>
-      <c r="C20" t="n">
-        <v>12104</v>
-      </c>
-      <c r="D20" t="n">
-        <v>983</v>
-      </c>
-      <c r="E20" t="n">
-        <v>1024</v>
-      </c>
-      <c r="F20" t="n">
-        <v>112</v>
-      </c>
-      <c r="G20" t="n">
-        <v>123</v>
-      </c>
-      <c r="H20" t="n">
-        <v>204.4</v>
-      </c>
-      <c r="I20" t="n">
-        <v>125.2</v>
-      </c>
-      <c r="J20" t="n">
         <v>38</v>
       </c>
     </row>

</xml_diff>